<commit_message>
Updated change history tab
Updated change history to reflect previous commit (forgot to do it for that commit)
</commit_message>
<xml_diff>
--- a/CPU Design/L1IsSequences.xlsx
+++ b/CPU Design/L1IsSequences.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="103" windowWidth="14803" windowHeight="8014"/>
+    <workbookView xWindow="240" yWindow="103" windowWidth="14803" windowHeight="8014" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sequences" sheetId="4" r:id="rId1"/>
@@ -579,7 +579,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4648" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4649" uniqueCount="234">
   <si>
     <t>STEP</t>
   </si>
@@ -1303,6 +1303,9 @@
   </si>
   <si>
     <t>Most of the signals are "active low", a few are "active high"</t>
+  </si>
+  <si>
+    <t>Changed all selects and SEQ_END from active high to active low.</t>
   </si>
 </sst>
 </file>
@@ -17105,7 +17108,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.6"/>
   <cols>
     <col min="1" max="1" width="9.3046875" style="17" customWidth="1"/>
@@ -17156,6 +17159,14 @@
         <v>229</v>
       </c>
     </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="16">
+        <v>46207</v>
+      </c>
+      <c r="B8" t="s">
+        <v>233</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>